<commit_message>
chore: delete excel columns (defaults only)
</commit_message>
<xml_diff>
--- a/KR_Stocks_ETF.xlsx
+++ b/KR_Stocks_ETF.xlsx
@@ -6905,7 +6905,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BM19"/>
+  <dimension ref="A1:AR19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -7196,111 +7196,6 @@
           <t>20251226</t>
         </is>
       </c>
-      <c r="AS1" s="1" t="inlineStr">
-        <is>
-          <t>20251201</t>
-        </is>
-      </c>
-      <c r="AT1" s="1" t="inlineStr">
-        <is>
-          <t>20251202</t>
-        </is>
-      </c>
-      <c r="AU1" s="1" t="inlineStr">
-        <is>
-          <t>20251203</t>
-        </is>
-      </c>
-      <c r="AV1" s="1" t="inlineStr">
-        <is>
-          <t>20251204</t>
-        </is>
-      </c>
-      <c r="AW1" s="1" t="inlineStr">
-        <is>
-          <t>20251205</t>
-        </is>
-      </c>
-      <c r="AX1" s="1" t="inlineStr">
-        <is>
-          <t>20251208</t>
-        </is>
-      </c>
-      <c r="AY1" s="1" t="inlineStr">
-        <is>
-          <t>20251209</t>
-        </is>
-      </c>
-      <c r="AZ1" s="1" t="inlineStr">
-        <is>
-          <t>20251210</t>
-        </is>
-      </c>
-      <c r="BA1" s="1" t="inlineStr">
-        <is>
-          <t>20251211</t>
-        </is>
-      </c>
-      <c r="BB1" s="1" t="inlineStr">
-        <is>
-          <t>20251212</t>
-        </is>
-      </c>
-      <c r="BC1" s="1" t="inlineStr">
-        <is>
-          <t>20251215</t>
-        </is>
-      </c>
-      <c r="BD1" s="1" t="inlineStr">
-        <is>
-          <t>20251216</t>
-        </is>
-      </c>
-      <c r="BE1" s="1" t="inlineStr">
-        <is>
-          <t>20251217</t>
-        </is>
-      </c>
-      <c r="BF1" s="1" t="inlineStr">
-        <is>
-          <t>20251218</t>
-        </is>
-      </c>
-      <c r="BG1" s="1" t="inlineStr">
-        <is>
-          <t>20251219</t>
-        </is>
-      </c>
-      <c r="BH1" s="1" t="inlineStr">
-        <is>
-          <t>20251222</t>
-        </is>
-      </c>
-      <c r="BI1" s="1" t="inlineStr">
-        <is>
-          <t>20251223</t>
-        </is>
-      </c>
-      <c r="BJ1" s="1" t="inlineStr">
-        <is>
-          <t>20251224</t>
-        </is>
-      </c>
-      <c r="BK1" s="1" t="inlineStr">
-        <is>
-          <t>20251226</t>
-        </is>
-      </c>
-      <c r="BL1" s="1" t="inlineStr">
-        <is>
-          <t>20251229</t>
-        </is>
-      </c>
-      <c r="BM1" s="1" t="inlineStr">
-        <is>
-          <t>20251230</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -7439,69 +7334,6 @@
       <c r="AR2" t="n">
         <v>15.38</v>
       </c>
-      <c r="AS2" t="n">
-        <v>645.79</v>
-      </c>
-      <c r="AT2" t="n">
-        <v>645.46</v>
-      </c>
-      <c r="AU2" t="n">
-        <v>626.3099999999999</v>
-      </c>
-      <c r="AV2" t="n">
-        <v>605.24</v>
-      </c>
-      <c r="AW2" t="n">
-        <v>529.66</v>
-      </c>
-      <c r="AX2" t="n">
-        <v>485.39</v>
-      </c>
-      <c r="AY2" t="n">
-        <v>399.28</v>
-      </c>
-      <c r="AZ2" t="n">
-        <v>393.37</v>
-      </c>
-      <c r="BA2" t="n">
-        <v>400.51</v>
-      </c>
-      <c r="BB2" t="n">
-        <v>409.79</v>
-      </c>
-      <c r="BC2" t="n">
-        <v>396.06</v>
-      </c>
-      <c r="BD2" t="n">
-        <v>405.58</v>
-      </c>
-      <c r="BE2" t="n">
-        <v>459.55</v>
-      </c>
-      <c r="BF2" t="n">
-        <v>485.11</v>
-      </c>
-      <c r="BG2" t="n">
-        <v>486.59</v>
-      </c>
-      <c r="BH2" t="n">
-        <v>518.64</v>
-      </c>
-      <c r="BI2" t="n">
-        <v>574.16</v>
-      </c>
-      <c r="BJ2" t="n">
-        <v>593.91</v>
-      </c>
-      <c r="BK2" t="n">
-        <v>595.36</v>
-      </c>
-      <c r="BL2" t="n">
-        <v>577.78</v>
-      </c>
-      <c r="BM2" t="n">
-        <v>547.09</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -7640,69 +7472,6 @@
       <c r="AR3" t="n">
         <v>-30.02</v>
       </c>
-      <c r="AS3" t="n">
-        <v>2299.56</v>
-      </c>
-      <c r="AT3" t="n">
-        <v>2173.53</v>
-      </c>
-      <c r="AU3" t="n">
-        <v>2155.48</v>
-      </c>
-      <c r="AV3" t="n">
-        <v>2090.2</v>
-      </c>
-      <c r="AW3" t="n">
-        <v>2089.1</v>
-      </c>
-      <c r="AX3" t="n">
-        <v>2063.38</v>
-      </c>
-      <c r="AY3" t="n">
-        <v>1938.42</v>
-      </c>
-      <c r="AZ3" t="n">
-        <v>1824.92</v>
-      </c>
-      <c r="BA3" t="n">
-        <v>1685.63</v>
-      </c>
-      <c r="BB3" t="n">
-        <v>1706.19</v>
-      </c>
-      <c r="BC3" t="n">
-        <v>1609.14</v>
-      </c>
-      <c r="BD3" t="n">
-        <v>1661</v>
-      </c>
-      <c r="BE3" t="n">
-        <v>1650.25</v>
-      </c>
-      <c r="BF3" t="n">
-        <v>1652.07</v>
-      </c>
-      <c r="BG3" t="n">
-        <v>1436.26</v>
-      </c>
-      <c r="BH3" t="n">
-        <v>1273.33</v>
-      </c>
-      <c r="BI3" t="n">
-        <v>1176.69</v>
-      </c>
-      <c r="BJ3" t="n">
-        <v>1118.28</v>
-      </c>
-      <c r="BK3" t="n">
-        <v>1235.59</v>
-      </c>
-      <c r="BL3" t="n">
-        <v>1442.86</v>
-      </c>
-      <c r="BM3" t="n">
-        <v>1666.41</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -7841,69 +7610,6 @@
       <c r="AR4" t="n">
         <v>12.89</v>
       </c>
-      <c r="AS4" t="n">
-        <v>741.65</v>
-      </c>
-      <c r="AT4" t="n">
-        <v>765.83</v>
-      </c>
-      <c r="AU4" t="n">
-        <v>753.1900000000001</v>
-      </c>
-      <c r="AV4" t="n">
-        <v>720.38</v>
-      </c>
-      <c r="AW4" t="n">
-        <v>648.59</v>
-      </c>
-      <c r="AX4" t="n">
-        <v>582.86</v>
-      </c>
-      <c r="AY4" t="n">
-        <v>449.84</v>
-      </c>
-      <c r="AZ4" t="n">
-        <v>449.02</v>
-      </c>
-      <c r="BA4" t="n">
-        <v>454.9</v>
-      </c>
-      <c r="BB4" t="n">
-        <v>487.83</v>
-      </c>
-      <c r="BC4" t="n">
-        <v>504.11</v>
-      </c>
-      <c r="BD4" t="n">
-        <v>524.1799999999999</v>
-      </c>
-      <c r="BE4" t="n">
-        <v>576.85</v>
-      </c>
-      <c r="BF4" t="n">
-        <v>587.75</v>
-      </c>
-      <c r="BG4" t="n">
-        <v>584.8099999999999</v>
-      </c>
-      <c r="BH4" t="n">
-        <v>605.08</v>
-      </c>
-      <c r="BI4" t="n">
-        <v>636.66</v>
-      </c>
-      <c r="BJ4" t="n">
-        <v>672.98</v>
-      </c>
-      <c r="BK4" t="n">
-        <v>687.22</v>
-      </c>
-      <c r="BL4" t="n">
-        <v>629.62</v>
-      </c>
-      <c r="BM4" t="n">
-        <v>561.4400000000001</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -8042,69 +7748,6 @@
       <c r="AR5" t="n">
         <v>-7.01</v>
       </c>
-      <c r="AS5" t="n">
-        <v>538.55</v>
-      </c>
-      <c r="AT5" t="n">
-        <v>492.53</v>
-      </c>
-      <c r="AU5" t="n">
-        <v>487.68</v>
-      </c>
-      <c r="AV5" t="n">
-        <v>473.21</v>
-      </c>
-      <c r="AW5" t="n">
-        <v>474.24</v>
-      </c>
-      <c r="AX5" t="n">
-        <v>467.85</v>
-      </c>
-      <c r="AY5" t="n">
-        <v>443.88</v>
-      </c>
-      <c r="AZ5" t="n">
-        <v>406.61</v>
-      </c>
-      <c r="BA5" t="n">
-        <v>369.26</v>
-      </c>
-      <c r="BB5" t="n">
-        <v>368.71</v>
-      </c>
-      <c r="BC5" t="n">
-        <v>347.38</v>
-      </c>
-      <c r="BD5" t="n">
-        <v>414.77</v>
-      </c>
-      <c r="BE5" t="n">
-        <v>420.64</v>
-      </c>
-      <c r="BF5" t="n">
-        <v>432.51</v>
-      </c>
-      <c r="BG5" t="n">
-        <v>429.24</v>
-      </c>
-      <c r="BH5" t="n">
-        <v>406.53</v>
-      </c>
-      <c r="BI5" t="n">
-        <v>408.7</v>
-      </c>
-      <c r="BJ5" t="n">
-        <v>411.25</v>
-      </c>
-      <c r="BK5" t="n">
-        <v>408.22</v>
-      </c>
-      <c r="BL5" t="n">
-        <v>416</v>
-      </c>
-      <c r="BM5" t="n">
-        <v>429.46</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -8243,69 +7886,6 @@
       <c r="AR6" t="n">
         <v>-22.11</v>
       </c>
-      <c r="AS6" t="n">
-        <v>522.97</v>
-      </c>
-      <c r="AT6" t="n">
-        <v>502.98</v>
-      </c>
-      <c r="AU6" t="n">
-        <v>506.77</v>
-      </c>
-      <c r="AV6" t="n">
-        <v>504.42</v>
-      </c>
-      <c r="AW6" t="n">
-        <v>503.05</v>
-      </c>
-      <c r="AX6" t="n">
-        <v>514.16</v>
-      </c>
-      <c r="AY6" t="n">
-        <v>505.93</v>
-      </c>
-      <c r="AZ6" t="n">
-        <v>503.9</v>
-      </c>
-      <c r="BA6" t="n">
-        <v>496.69</v>
-      </c>
-      <c r="BB6" t="n">
-        <v>496.61</v>
-      </c>
-      <c r="BC6" t="n">
-        <v>477.43</v>
-      </c>
-      <c r="BD6" t="n">
-        <v>494.38</v>
-      </c>
-      <c r="BE6" t="n">
-        <v>486.78</v>
-      </c>
-      <c r="BF6" t="n">
-        <v>491.45</v>
-      </c>
-      <c r="BG6" t="n">
-        <v>428.16</v>
-      </c>
-      <c r="BH6" t="n">
-        <v>362.93</v>
-      </c>
-      <c r="BI6" t="n">
-        <v>342.84</v>
-      </c>
-      <c r="BJ6" t="n">
-        <v>337.45</v>
-      </c>
-      <c r="BK6" t="n">
-        <v>366.92</v>
-      </c>
-      <c r="BL6" t="n">
-        <v>418.45</v>
-      </c>
-      <c r="BM6" t="n">
-        <v>471.64</v>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -8444,69 +8024,6 @@
       <c r="AR7" t="n">
         <v>-29.72</v>
       </c>
-      <c r="AS7" t="n">
-        <v>613.1</v>
-      </c>
-      <c r="AT7" t="n">
-        <v>584.49</v>
-      </c>
-      <c r="AU7" t="n">
-        <v>599.25</v>
-      </c>
-      <c r="AV7" t="n">
-        <v>599.4299999999999</v>
-      </c>
-      <c r="AW7" t="n">
-        <v>612.26</v>
-      </c>
-      <c r="AX7" t="n">
-        <v>639.23</v>
-      </c>
-      <c r="AY7" t="n">
-        <v>643.13</v>
-      </c>
-      <c r="AZ7" t="n">
-        <v>662.4400000000001</v>
-      </c>
-      <c r="BA7" t="n">
-        <v>667.24</v>
-      </c>
-      <c r="BB7" t="n">
-        <v>679.04</v>
-      </c>
-      <c r="BC7" t="n">
-        <v>679.89</v>
-      </c>
-      <c r="BD7" t="n">
-        <v>664.88</v>
-      </c>
-      <c r="BE7" t="n">
-        <v>640.21</v>
-      </c>
-      <c r="BF7" t="n">
-        <v>631.26</v>
-      </c>
-      <c r="BG7" t="n">
-        <v>518.92</v>
-      </c>
-      <c r="BH7" t="n">
-        <v>427.02</v>
-      </c>
-      <c r="BI7" t="n">
-        <v>371.28</v>
-      </c>
-      <c r="BJ7" t="n">
-        <v>364.46</v>
-      </c>
-      <c r="BK7" t="n">
-        <v>410.92</v>
-      </c>
-      <c r="BL7" t="n">
-        <v>484.03</v>
-      </c>
-      <c r="BM7" t="n">
-        <v>555.38</v>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -8645,69 +8162,6 @@
       <c r="AR8" t="n">
         <v>-21.24</v>
       </c>
-      <c r="AS8" t="n">
-        <v>695.97</v>
-      </c>
-      <c r="AT8" t="n">
-        <v>660.11</v>
-      </c>
-      <c r="AU8" t="n">
-        <v>658.1</v>
-      </c>
-      <c r="AV8" t="n">
-        <v>651.63</v>
-      </c>
-      <c r="AW8" t="n">
-        <v>652.0599999999999</v>
-      </c>
-      <c r="AX8" t="n">
-        <v>649.63</v>
-      </c>
-      <c r="AY8" t="n">
-        <v>616.5599999999999</v>
-      </c>
-      <c r="AZ8" t="n">
-        <v>588.03</v>
-      </c>
-      <c r="BA8" t="n">
-        <v>541.03</v>
-      </c>
-      <c r="BB8" t="n">
-        <v>553.79</v>
-      </c>
-      <c r="BC8" t="n">
-        <v>524.87</v>
-      </c>
-      <c r="BD8" t="n">
-        <v>538.9</v>
-      </c>
-      <c r="BE8" t="n">
-        <v>534.54</v>
-      </c>
-      <c r="BF8" t="n">
-        <v>534.58</v>
-      </c>
-      <c r="BG8" t="n">
-        <v>464.25</v>
-      </c>
-      <c r="BH8" t="n">
-        <v>402.72</v>
-      </c>
-      <c r="BI8" t="n">
-        <v>378.65</v>
-      </c>
-      <c r="BJ8" t="n">
-        <v>384.23</v>
-      </c>
-      <c r="BK8" t="n">
-        <v>441.75</v>
-      </c>
-      <c r="BL8" t="n">
-        <v>539.3200000000001</v>
-      </c>
-      <c r="BM8" t="n">
-        <v>632.08</v>
-      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -8846,69 +8300,6 @@
       <c r="AR9" t="n">
         <v>12.29</v>
       </c>
-      <c r="AS9" t="n">
-        <v>125.35</v>
-      </c>
-      <c r="AT9" t="n">
-        <v>120.99</v>
-      </c>
-      <c r="AU9" t="n">
-        <v>120.58</v>
-      </c>
-      <c r="AV9" t="n">
-        <v>120.22</v>
-      </c>
-      <c r="AW9" t="n">
-        <v>120.47</v>
-      </c>
-      <c r="AX9" t="n">
-        <v>120.32</v>
-      </c>
-      <c r="AY9" t="n">
-        <v>118.18</v>
-      </c>
-      <c r="AZ9" t="n">
-        <v>109.82</v>
-      </c>
-      <c r="BA9" t="n">
-        <v>87.8</v>
-      </c>
-      <c r="BB9" t="n">
-        <v>82.48</v>
-      </c>
-      <c r="BC9" t="n">
-        <v>76.67</v>
-      </c>
-      <c r="BD9" t="n">
-        <v>78.52</v>
-      </c>
-      <c r="BE9" t="n">
-        <v>79.45</v>
-      </c>
-      <c r="BF9" t="n">
-        <v>91.86</v>
-      </c>
-      <c r="BG9" t="n">
-        <v>102.65</v>
-      </c>
-      <c r="BH9" t="n">
-        <v>105.63</v>
-      </c>
-      <c r="BI9" t="n">
-        <v>109.27</v>
-      </c>
-      <c r="BJ9" t="n">
-        <v>113.27</v>
-      </c>
-      <c r="BK9" t="n">
-        <v>119.62</v>
-      </c>
-      <c r="BL9" t="n">
-        <v>126.26</v>
-      </c>
-      <c r="BM9" t="n">
-        <v>136.94</v>
-      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -9047,69 +8438,6 @@
       <c r="AR10" t="n">
         <v>8.720000000000001</v>
       </c>
-      <c r="AS10" t="n">
-        <v>516.12</v>
-      </c>
-      <c r="AT10" t="n">
-        <v>467.23</v>
-      </c>
-      <c r="AU10" t="n">
-        <v>480.23</v>
-      </c>
-      <c r="AV10" t="n">
-        <v>474.84</v>
-      </c>
-      <c r="AW10" t="n">
-        <v>464.08</v>
-      </c>
-      <c r="AX10" t="n">
-        <v>464.08</v>
-      </c>
-      <c r="AY10" t="n">
-        <v>463.43</v>
-      </c>
-      <c r="AZ10" t="n">
-        <v>459.17</v>
-      </c>
-      <c r="BA10" t="n">
-        <v>448.36</v>
-      </c>
-      <c r="BB10" t="n">
-        <v>442.01</v>
-      </c>
-      <c r="BC10" t="n">
-        <v>438.69</v>
-      </c>
-      <c r="BD10" t="n">
-        <v>497.54</v>
-      </c>
-      <c r="BE10" t="n">
-        <v>510.01</v>
-      </c>
-      <c r="BF10" t="n">
-        <v>555.96</v>
-      </c>
-      <c r="BG10" t="n">
-        <v>558.1799999999999</v>
-      </c>
-      <c r="BH10" t="n">
-        <v>527.25</v>
-      </c>
-      <c r="BI10" t="n">
-        <v>533.13</v>
-      </c>
-      <c r="BJ10" t="n">
-        <v>545.4299999999999</v>
-      </c>
-      <c r="BK10" t="n">
-        <v>539.1900000000001</v>
-      </c>
-      <c r="BL10" t="n">
-        <v>522.64</v>
-      </c>
-      <c r="BM10" t="n">
-        <v>503.14</v>
-      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -9248,69 +8576,6 @@
       <c r="AR11" t="n">
         <v>-3.13</v>
       </c>
-      <c r="AS11" t="n">
-        <v>202.62</v>
-      </c>
-      <c r="AT11" t="n">
-        <v>197.34</v>
-      </c>
-      <c r="AU11" t="n">
-        <v>198.21</v>
-      </c>
-      <c r="AV11" t="n">
-        <v>197.43</v>
-      </c>
-      <c r="AW11" t="n">
-        <v>199.08</v>
-      </c>
-      <c r="AX11" t="n">
-        <v>227.13</v>
-      </c>
-      <c r="AY11" t="n">
-        <v>255.36</v>
-      </c>
-      <c r="AZ11" t="n">
-        <v>272</v>
-      </c>
-      <c r="BA11" t="n">
-        <v>270.08</v>
-      </c>
-      <c r="BB11" t="n">
-        <v>281.11</v>
-      </c>
-      <c r="BC11" t="n">
-        <v>291.58</v>
-      </c>
-      <c r="BD11" t="n">
-        <v>287.96</v>
-      </c>
-      <c r="BE11" t="n">
-        <v>283.89</v>
-      </c>
-      <c r="BF11" t="n">
-        <v>287.89</v>
-      </c>
-      <c r="BG11" t="n">
-        <v>279.21</v>
-      </c>
-      <c r="BH11" t="n">
-        <v>252.58</v>
-      </c>
-      <c r="BI11" t="n">
-        <v>229.35</v>
-      </c>
-      <c r="BJ11" t="n">
-        <v>232.75</v>
-      </c>
-      <c r="BK11" t="n">
-        <v>236.83</v>
-      </c>
-      <c r="BL11" t="n">
-        <v>239.07</v>
-      </c>
-      <c r="BM11" t="n">
-        <v>258.52</v>
-      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -9449,69 +8714,6 @@
       <c r="AR12" t="n">
         <v>-1.83</v>
       </c>
-      <c r="AS12" t="n">
-        <v>242.38</v>
-      </c>
-      <c r="AT12" t="n">
-        <v>234.69</v>
-      </c>
-      <c r="AU12" t="n">
-        <v>233.74</v>
-      </c>
-      <c r="AV12" t="n">
-        <v>229.75</v>
-      </c>
-      <c r="AW12" t="n">
-        <v>232.36</v>
-      </c>
-      <c r="AX12" t="n">
-        <v>271.02</v>
-      </c>
-      <c r="AY12" t="n">
-        <v>306.45</v>
-      </c>
-      <c r="AZ12" t="n">
-        <v>327.33</v>
-      </c>
-      <c r="BA12" t="n">
-        <v>328.87</v>
-      </c>
-      <c r="BB12" t="n">
-        <v>343.38</v>
-      </c>
-      <c r="BC12" t="n">
-        <v>358.04</v>
-      </c>
-      <c r="BD12" t="n">
-        <v>353.7</v>
-      </c>
-      <c r="BE12" t="n">
-        <v>347.62</v>
-      </c>
-      <c r="BF12" t="n">
-        <v>350.42</v>
-      </c>
-      <c r="BG12" t="n">
-        <v>341.49</v>
-      </c>
-      <c r="BH12" t="n">
-        <v>312.62</v>
-      </c>
-      <c r="BI12" t="n">
-        <v>283.31</v>
-      </c>
-      <c r="BJ12" t="n">
-        <v>286.28</v>
-      </c>
-      <c r="BK12" t="n">
-        <v>290.77</v>
-      </c>
-      <c r="BL12" t="n">
-        <v>295.19</v>
-      </c>
-      <c r="BM12" t="n">
-        <v>322.46</v>
-      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -9650,69 +8852,6 @@
       <c r="AR13" t="n">
         <v>-8.07</v>
       </c>
-      <c r="AS13" t="n">
-        <v>260.33</v>
-      </c>
-      <c r="AT13" t="n">
-        <v>250.73</v>
-      </c>
-      <c r="AU13" t="n">
-        <v>250.25</v>
-      </c>
-      <c r="AV13" t="n">
-        <v>246.23</v>
-      </c>
-      <c r="AW13" t="n">
-        <v>251.08</v>
-      </c>
-      <c r="AX13" t="n">
-        <v>302.57</v>
-      </c>
-      <c r="AY13" t="n">
-        <v>348.5</v>
-      </c>
-      <c r="AZ13" t="n">
-        <v>379.25</v>
-      </c>
-      <c r="BA13" t="n">
-        <v>391.93</v>
-      </c>
-      <c r="BB13" t="n">
-        <v>411.32</v>
-      </c>
-      <c r="BC13" t="n">
-        <v>430.25</v>
-      </c>
-      <c r="BD13" t="n">
-        <v>424.14</v>
-      </c>
-      <c r="BE13" t="n">
-        <v>415.82</v>
-      </c>
-      <c r="BF13" t="n">
-        <v>413.12</v>
-      </c>
-      <c r="BG13" t="n">
-        <v>396.3</v>
-      </c>
-      <c r="BH13" t="n">
-        <v>358.39</v>
-      </c>
-      <c r="BI13" t="n">
-        <v>319.15</v>
-      </c>
-      <c r="BJ13" t="n">
-        <v>314.34</v>
-      </c>
-      <c r="BK13" t="n">
-        <v>309.93</v>
-      </c>
-      <c r="BL13" t="n">
-        <v>305</v>
-      </c>
-      <c r="BM13" t="n">
-        <v>326.23</v>
-      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -9851,69 +8990,6 @@
       <c r="AR14" t="n">
         <v>9.380000000000001</v>
       </c>
-      <c r="AS14" t="n">
-        <v>150.35</v>
-      </c>
-      <c r="AT14" t="n">
-        <v>143.29</v>
-      </c>
-      <c r="AU14" t="n">
-        <v>141.2</v>
-      </c>
-      <c r="AV14" t="n">
-        <v>138.61</v>
-      </c>
-      <c r="AW14" t="n">
-        <v>138.52</v>
-      </c>
-      <c r="AX14" t="n">
-        <v>140.39</v>
-      </c>
-      <c r="AY14" t="n">
-        <v>140.12</v>
-      </c>
-      <c r="AZ14" t="n">
-        <v>135.9</v>
-      </c>
-      <c r="BA14" t="n">
-        <v>115.86</v>
-      </c>
-      <c r="BB14" t="n">
-        <v>113.8</v>
-      </c>
-      <c r="BC14" t="n">
-        <v>112.21</v>
-      </c>
-      <c r="BD14" t="n">
-        <v>112.87</v>
-      </c>
-      <c r="BE14" t="n">
-        <v>113.02</v>
-      </c>
-      <c r="BF14" t="n">
-        <v>125.49</v>
-      </c>
-      <c r="BG14" t="n">
-        <v>133.31</v>
-      </c>
-      <c r="BH14" t="n">
-        <v>131.14</v>
-      </c>
-      <c r="BI14" t="n">
-        <v>131.22</v>
-      </c>
-      <c r="BJ14" t="n">
-        <v>137.06</v>
-      </c>
-      <c r="BK14" t="n">
-        <v>145.2</v>
-      </c>
-      <c r="BL14" t="n">
-        <v>152.5</v>
-      </c>
-      <c r="BM14" t="n">
-        <v>165.68</v>
-      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -10052,69 +9128,6 @@
       <c r="AR15" t="n">
         <v>-24</v>
       </c>
-      <c r="AS15" t="n">
-        <v>1228.63</v>
-      </c>
-      <c r="AT15" t="n">
-        <v>1259.82</v>
-      </c>
-      <c r="AU15" t="n">
-        <v>1256.74</v>
-      </c>
-      <c r="AV15" t="n">
-        <v>1234.86</v>
-      </c>
-      <c r="AW15" t="n">
-        <v>1107.2</v>
-      </c>
-      <c r="AX15" t="n">
-        <v>943.66</v>
-      </c>
-      <c r="AY15" t="n">
-        <v>650.0599999999999</v>
-      </c>
-      <c r="AZ15" t="n">
-        <v>598.54</v>
-      </c>
-      <c r="BA15" t="n">
-        <v>571.54</v>
-      </c>
-      <c r="BB15" t="n">
-        <v>560.66</v>
-      </c>
-      <c r="BC15" t="n">
-        <v>561.76</v>
-      </c>
-      <c r="BD15" t="n">
-        <v>556.28</v>
-      </c>
-      <c r="BE15" t="n">
-        <v>559.16</v>
-      </c>
-      <c r="BF15" t="n">
-        <v>582.75</v>
-      </c>
-      <c r="BG15" t="n">
-        <v>584.22</v>
-      </c>
-      <c r="BH15" t="n">
-        <v>586.79</v>
-      </c>
-      <c r="BI15" t="n">
-        <v>580.71</v>
-      </c>
-      <c r="BJ15" t="n">
-        <v>602.4400000000001</v>
-      </c>
-      <c r="BK15" t="n">
-        <v>601.85</v>
-      </c>
-      <c r="BL15" t="n">
-        <v>585.6799999999999</v>
-      </c>
-      <c r="BM15" t="n">
-        <v>543.92</v>
-      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -10253,69 +9266,6 @@
       <c r="AR16" t="n">
         <v>1.94</v>
       </c>
-      <c r="AS16" t="n">
-        <v>473.01</v>
-      </c>
-      <c r="AT16" t="n">
-        <v>444.08</v>
-      </c>
-      <c r="AU16" t="n">
-        <v>434.67</v>
-      </c>
-      <c r="AV16" t="n">
-        <v>422.92</v>
-      </c>
-      <c r="AW16" t="n">
-        <v>423.8</v>
-      </c>
-      <c r="AX16" t="n">
-        <v>458.44</v>
-      </c>
-      <c r="AY16" t="n">
-        <v>489.93</v>
-      </c>
-      <c r="AZ16" t="n">
-        <v>501.78</v>
-      </c>
-      <c r="BA16" t="n">
-        <v>477.47</v>
-      </c>
-      <c r="BB16" t="n">
-        <v>494.73</v>
-      </c>
-      <c r="BC16" t="n">
-        <v>511.45</v>
-      </c>
-      <c r="BD16" t="n">
-        <v>508.1</v>
-      </c>
-      <c r="BE16" t="n">
-        <v>500.44</v>
-      </c>
-      <c r="BF16" t="n">
-        <v>517.54</v>
-      </c>
-      <c r="BG16" t="n">
-        <v>517.54</v>
-      </c>
-      <c r="BH16" t="n">
-        <v>484.28</v>
-      </c>
-      <c r="BI16" t="n">
-        <v>458.77</v>
-      </c>
-      <c r="BJ16" t="n">
-        <v>470.28</v>
-      </c>
-      <c r="BK16" t="n">
-        <v>488.01</v>
-      </c>
-      <c r="BL16" t="n">
-        <v>502.23</v>
-      </c>
-      <c r="BM16" t="n">
-        <v>548.13</v>
-      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -10454,69 +9404,6 @@
       <c r="AR17" t="n">
         <v>-0.84</v>
       </c>
-      <c r="AS17" t="n">
-        <v>310.75</v>
-      </c>
-      <c r="AT17" t="n">
-        <v>300.76</v>
-      </c>
-      <c r="AU17" t="n">
-        <v>296.58</v>
-      </c>
-      <c r="AV17" t="n">
-        <v>291.51</v>
-      </c>
-      <c r="AW17" t="n">
-        <v>291.53</v>
-      </c>
-      <c r="AX17" t="n">
-        <v>309.76</v>
-      </c>
-      <c r="AY17" t="n">
-        <v>326.92</v>
-      </c>
-      <c r="AZ17" t="n">
-        <v>332.96</v>
-      </c>
-      <c r="BA17" t="n">
-        <v>305.22</v>
-      </c>
-      <c r="BB17" t="n">
-        <v>310.05</v>
-      </c>
-      <c r="BC17" t="n">
-        <v>317.75</v>
-      </c>
-      <c r="BD17" t="n">
-        <v>316.64</v>
-      </c>
-      <c r="BE17" t="n">
-        <v>312.4</v>
-      </c>
-      <c r="BF17" t="n">
-        <v>324.58</v>
-      </c>
-      <c r="BG17" t="n">
-        <v>325.21</v>
-      </c>
-      <c r="BH17" t="n">
-        <v>302.89</v>
-      </c>
-      <c r="BI17" t="n">
-        <v>282.64</v>
-      </c>
-      <c r="BJ17" t="n">
-        <v>291.92</v>
-      </c>
-      <c r="BK17" t="n">
-        <v>306.24</v>
-      </c>
-      <c r="BL17" t="n">
-        <v>320.15</v>
-      </c>
-      <c r="BM17" t="n">
-        <v>353.21</v>
-      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -10655,69 +9542,6 @@
       <c r="AR18" t="n">
         <v>3.33</v>
       </c>
-      <c r="AS18" t="n">
-        <v>626.28</v>
-      </c>
-      <c r="AT18" t="n">
-        <v>636.1900000000001</v>
-      </c>
-      <c r="AU18" t="n">
-        <v>630.64</v>
-      </c>
-      <c r="AV18" t="n">
-        <v>621.76</v>
-      </c>
-      <c r="AW18" t="n">
-        <v>550.73</v>
-      </c>
-      <c r="AX18" t="n">
-        <v>553.5599999999999</v>
-      </c>
-      <c r="AY18" t="n">
-        <v>558.8</v>
-      </c>
-      <c r="AZ18" t="n">
-        <v>566.0700000000001</v>
-      </c>
-      <c r="BA18" t="n">
-        <v>568.14</v>
-      </c>
-      <c r="BB18" t="n">
-        <v>507.01</v>
-      </c>
-      <c r="BC18" t="n">
-        <v>528.0599999999999</v>
-      </c>
-      <c r="BD18" t="n">
-        <v>605.0599999999999</v>
-      </c>
-      <c r="BE18" t="n">
-        <v>627.87</v>
-      </c>
-      <c r="BF18" t="n">
-        <v>674.0700000000001</v>
-      </c>
-      <c r="BG18" t="n">
-        <v>674.5</v>
-      </c>
-      <c r="BH18" t="n">
-        <v>645.4400000000001</v>
-      </c>
-      <c r="BI18" t="n">
-        <v>652.11</v>
-      </c>
-      <c r="BJ18" t="n">
-        <v>647.17</v>
-      </c>
-      <c r="BK18" t="n">
-        <v>625.4400000000001</v>
-      </c>
-      <c r="BL18" t="n">
-        <v>594.71</v>
-      </c>
-      <c r="BM18" t="n">
-        <v>579.6900000000001</v>
-      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -10855,69 +9679,6 @@
       </c>
       <c r="AR19" t="n">
         <v>-39.13</v>
-      </c>
-      <c r="AS19" t="n">
-        <v>868</v>
-      </c>
-      <c r="AT19" t="n">
-        <v>893.52</v>
-      </c>
-      <c r="AU19" t="n">
-        <v>887.01</v>
-      </c>
-      <c r="AV19" t="n">
-        <v>864.12</v>
-      </c>
-      <c r="AW19" t="n">
-        <v>775.66</v>
-      </c>
-      <c r="AX19" t="n">
-        <v>649.9400000000001</v>
-      </c>
-      <c r="AY19" t="n">
-        <v>441.38</v>
-      </c>
-      <c r="AZ19" t="n">
-        <v>424.12</v>
-      </c>
-      <c r="BA19" t="n">
-        <v>418.55</v>
-      </c>
-      <c r="BB19" t="n">
-        <v>417.46</v>
-      </c>
-      <c r="BC19" t="n">
-        <v>419.76</v>
-      </c>
-      <c r="BD19" t="n">
-        <v>416.94</v>
-      </c>
-      <c r="BE19" t="n">
-        <v>409.53</v>
-      </c>
-      <c r="BF19" t="n">
-        <v>415.35</v>
-      </c>
-      <c r="BG19" t="n">
-        <v>410.12</v>
-      </c>
-      <c r="BH19" t="n">
-        <v>391.44</v>
-      </c>
-      <c r="BI19" t="n">
-        <v>342.28</v>
-      </c>
-      <c r="BJ19" t="n">
-        <v>341.66</v>
-      </c>
-      <c r="BK19" t="n">
-        <v>333.84</v>
-      </c>
-      <c r="BL19" t="n">
-        <v>331.58</v>
-      </c>
-      <c r="BM19" t="n">
-        <v>300.88</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Recompute STD sheet (last 10 days)
</commit_message>
<xml_diff>
--- a/KR_Stocks_ETF.xlsx
+++ b/KR_Stocks_ETF.xlsx
@@ -6907,294 +6907,143 @@
   </sheetPr>
   <dimension ref="A1:AR19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="12" customWidth="1" min="15" max="15"/>
-    <col width="12" customWidth="1" min="16" max="16"/>
-    <col width="12" customWidth="1" min="17" max="17"/>
-    <col width="12" customWidth="1" min="18" max="18"/>
-    <col width="12" customWidth="1" min="19" max="19"/>
-    <col width="12" customWidth="1" min="20" max="20"/>
-    <col width="12" customWidth="1" min="21" max="21"/>
-    <col width="12" customWidth="1" min="22" max="22"/>
-    <col width="12" customWidth="1" min="23" max="23"/>
-    <col width="12" customWidth="1" min="24" max="24"/>
-    <col width="12" customWidth="1" min="25" max="25"/>
-    <col width="12" customWidth="1" min="26" max="26"/>
-    <col width="12" customWidth="1" min="27" max="27"/>
-    <col width="12" customWidth="1" min="28" max="28"/>
-    <col width="12" customWidth="1" min="29" max="29"/>
-    <col width="12" customWidth="1" min="30" max="30"/>
-    <col width="12" customWidth="1" min="31" max="31"/>
-    <col width="12" customWidth="1" min="32" max="32"/>
-    <col width="12" customWidth="1" min="33" max="33"/>
-    <col width="12" customWidth="1" min="34" max="34"/>
-    <col width="12" customWidth="1" min="35" max="35"/>
-    <col width="12" customWidth="1" min="36" max="36"/>
-    <col width="12" customWidth="1" min="37" max="37"/>
-    <col width="12" customWidth="1" min="38" max="38"/>
-    <col width="12" customWidth="1" min="39" max="39"/>
-    <col width="12" customWidth="1" min="40" max="40"/>
-    <col width="12" customWidth="1" min="41" max="41"/>
-    <col width="12" customWidth="1" min="42" max="42"/>
-    <col width="12" customWidth="1" min="43" max="43"/>
-    <col width="12" customWidth="1" min="44" max="44"/>
-    <col width="12" customWidth="1" min="45" max="45"/>
-    <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="12" customWidth="1" min="47" max="47"/>
-    <col width="12" customWidth="1" min="48" max="48"/>
-    <col width="12" customWidth="1" min="49" max="49"/>
-    <col width="12" customWidth="1" min="50" max="50"/>
-    <col width="12" customWidth="1" min="51" max="51"/>
-    <col width="12" customWidth="1" min="52" max="52"/>
-    <col width="12" customWidth="1" min="53" max="53"/>
-    <col width="12" customWidth="1" min="54" max="54"/>
-    <col width="12" customWidth="1" min="55" max="55"/>
-    <col width="12" customWidth="1" min="56" max="56"/>
-    <col width="12" customWidth="1" min="57" max="57"/>
-    <col width="12" customWidth="1" min="58" max="58"/>
-    <col width="12" customWidth="1" min="59" max="59"/>
-    <col width="12" customWidth="1" min="60" max="60"/>
-    <col width="12" customWidth="1" min="61" max="61"/>
-    <col width="12" customWidth="1" min="62" max="62"/>
-    <col width="12" customWidth="1" min="63" max="63"/>
-    <col width="12" customWidth="1" min="64" max="64"/>
-    <col width="12" customWidth="1" min="65" max="65"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>종목명</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>종목코드</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>20251029</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>20251030</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>20251031</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>20251103</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>20251104</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>20251105</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>20251106</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>20251107</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>20251110</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>20251111</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>20251112</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>20251113</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>20251114</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>20251117</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>20251118</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>20251119</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>20251120</t>
-        </is>
-      </c>
-      <c r="T1" s="1" t="inlineStr">
-        <is>
-          <t>20251121</t>
-        </is>
-      </c>
-      <c r="U1" s="1" t="inlineStr">
-        <is>
-          <t>20251124</t>
-        </is>
-      </c>
-      <c r="V1" s="1" t="inlineStr">
-        <is>
-          <t>20251125</t>
-        </is>
-      </c>
-      <c r="W1" s="1" t="inlineStr">
-        <is>
-          <t>20251126</t>
-        </is>
-      </c>
-      <c r="X1" s="1" t="inlineStr">
-        <is>
-          <t>20251127</t>
-        </is>
-      </c>
-      <c r="Y1" s="1" t="inlineStr">
-        <is>
-          <t>20251128</t>
-        </is>
-      </c>
-      <c r="Z1" s="1" t="inlineStr">
-        <is>
-          <t>20251201</t>
-        </is>
-      </c>
-      <c r="AA1" s="1" t="inlineStr">
-        <is>
-          <t>20251202</t>
-        </is>
-      </c>
-      <c r="AB1" s="1" t="inlineStr">
-        <is>
-          <t>20251203</t>
-        </is>
-      </c>
-      <c r="AC1" s="1" t="inlineStr">
-        <is>
-          <t>20251204</t>
-        </is>
-      </c>
-      <c r="AD1" s="1" t="inlineStr">
-        <is>
-          <t>20251205</t>
-        </is>
-      </c>
-      <c r="AE1" s="1" t="inlineStr">
-        <is>
-          <t>20251208</t>
-        </is>
-      </c>
-      <c r="AF1" s="1" t="inlineStr">
-        <is>
-          <t>20251209</t>
-        </is>
-      </c>
-      <c r="AG1" s="1" t="inlineStr">
-        <is>
-          <t>20251210</t>
-        </is>
-      </c>
-      <c r="AH1" s="1" t="inlineStr">
-        <is>
-          <t>20251211</t>
-        </is>
-      </c>
-      <c r="AI1" s="1" t="inlineStr">
-        <is>
-          <t>20251212</t>
-        </is>
-      </c>
-      <c r="AJ1" s="1" t="inlineStr">
-        <is>
-          <t>20251215</t>
-        </is>
-      </c>
-      <c r="AK1" s="1" t="inlineStr">
-        <is>
-          <t>20251216</t>
-        </is>
-      </c>
-      <c r="AL1" s="1" t="inlineStr">
-        <is>
-          <t>20251217</t>
-        </is>
-      </c>
-      <c r="AM1" s="1" t="inlineStr">
-        <is>
-          <t>20251218</t>
-        </is>
-      </c>
-      <c r="AN1" s="1" t="inlineStr">
-        <is>
-          <t>20251219</t>
-        </is>
-      </c>
-      <c r="AO1" s="1" t="inlineStr">
-        <is>
-          <t>20251222</t>
-        </is>
-      </c>
-      <c r="AP1" s="1" t="inlineStr">
-        <is>
-          <t>20251223</t>
-        </is>
-      </c>
-      <c r="AQ1" s="1" t="inlineStr">
-        <is>
-          <t>20251224</t>
-        </is>
-      </c>
-      <c r="AR1" s="1" t="inlineStr">
-        <is>
-          <t>20251226</t>
-        </is>
+      <c r="C1" t="n">
+        <v>20251029</v>
+      </c>
+      <c r="D1" t="n">
+        <v>20251030</v>
+      </c>
+      <c r="E1" t="n">
+        <v>20251031</v>
+      </c>
+      <c r="F1" t="n">
+        <v>20251103</v>
+      </c>
+      <c r="G1" t="n">
+        <v>20251104</v>
+      </c>
+      <c r="H1" t="n">
+        <v>20251105</v>
+      </c>
+      <c r="I1" t="n">
+        <v>20251106</v>
+      </c>
+      <c r="J1" t="n">
+        <v>20251107</v>
+      </c>
+      <c r="K1" t="n">
+        <v>20251110</v>
+      </c>
+      <c r="L1" t="n">
+        <v>20251111</v>
+      </c>
+      <c r="M1" t="n">
+        <v>20251112</v>
+      </c>
+      <c r="N1" t="n">
+        <v>20251113</v>
+      </c>
+      <c r="O1" t="n">
+        <v>20251114</v>
+      </c>
+      <c r="P1" t="n">
+        <v>20251117</v>
+      </c>
+      <c r="Q1" t="n">
+        <v>20251118</v>
+      </c>
+      <c r="R1" t="n">
+        <v>20251119</v>
+      </c>
+      <c r="S1" t="n">
+        <v>20251120</v>
+      </c>
+      <c r="T1" t="n">
+        <v>20251121</v>
+      </c>
+      <c r="U1" t="n">
+        <v>20251124</v>
+      </c>
+      <c r="V1" t="n">
+        <v>20251125</v>
+      </c>
+      <c r="W1" t="n">
+        <v>20251126</v>
+      </c>
+      <c r="X1" t="n">
+        <v>20251127</v>
+      </c>
+      <c r="Y1" t="n">
+        <v>20251128</v>
+      </c>
+      <c r="Z1" t="n">
+        <v>20251201</v>
+      </c>
+      <c r="AA1" t="n">
+        <v>20251202</v>
+      </c>
+      <c r="AB1" t="n">
+        <v>20251203</v>
+      </c>
+      <c r="AC1" t="n">
+        <v>20251204</v>
+      </c>
+      <c r="AD1" t="n">
+        <v>20251205</v>
+      </c>
+      <c r="AE1" t="n">
+        <v>20251208</v>
+      </c>
+      <c r="AF1" t="n">
+        <v>20251209</v>
+      </c>
+      <c r="AG1" t="n">
+        <v>20251210</v>
+      </c>
+      <c r="AH1" t="n">
+        <v>20251211</v>
+      </c>
+      <c r="AI1" t="n">
+        <v>20251212</v>
+      </c>
+      <c r="AJ1" t="n">
+        <v>20251215</v>
+      </c>
+      <c r="AK1" t="n">
+        <v>20251216</v>
+      </c>
+      <c r="AL1" t="n">
+        <v>20251217</v>
+      </c>
+      <c r="AM1" t="n">
+        <v>20251218</v>
+      </c>
+      <c r="AN1" t="n">
+        <v>20251219</v>
+      </c>
+      <c r="AO1" t="n">
+        <v>20251222</v>
+      </c>
+      <c r="AP1" t="n">
+        <v>20251223</v>
+      </c>
+      <c r="AQ1" t="n">
+        <v>20251224</v>
+      </c>
+      <c r="AR1" t="n">
+        <v>20251226</v>
       </c>
     </row>
     <row r="2">
@@ -7205,7 +7054,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0000Z0</t>
+          <t>000000</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -9510,7 +9359,7 @@
         <v>-1.15</v>
       </c>
       <c r="AH18" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AI18" t="n">
         <v>-9.880000000000001</v>

</xml_diff>